<commit_message>
feat(5/16): Subpackage Free 카드 range, K-Wellness sub dedupe, 상품 description 일괄 정리본
- agent/product priceLabel: Subpackage markup=0 multi-variant은 'Free – $X' range 표시
- agent/product 모달 정렬: Subpackage Free만 asc(저가→고가), 그 외 desc 유지
- agent/admin product 페이지: K-Wellness subcategory 칩 이름 기준 dedupe (React key warning fix)
- data/product_descriptions.txt: v25 159개 description 정리본 (★ ▶ • 양식 통일, K-Wellness SPA #P-201~207는 보존, 오탈자 일괄 fix)
- data/scripts/reformat_descriptions.py: 재실행 가능 정리 스크립트 (force-add)
- notes/26.05.15: 5/16 후속 세션 + Hotel 큐레이션 가이드 + v25 audit 기록

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/products_master_v24.xlsx
+++ b/data/products_master_v24.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102FAB85-C45E-46C3-B71E-654138CE43C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE7A2E0-B921-4ED5-8DE2-0C012B5F0B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="K-Medical" sheetId="1" r:id="rId1"/>
@@ -16,22 +16,11 @@
     <sheet name="Subpackage" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3769" uniqueCount="974">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3801" uniqueCount="983">
   <si>
     <t>product_number</t>
   </si>
@@ -3104,9 +3093,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>(06351) 서울특별시 강남구 일원로 82 삼성서울병원</t>
-  </si>
-  <si>
     <t>#P-011</t>
   </si>
   <si>
@@ -3817,6 +3803,46 @@
   </si>
   <si>
     <t>#P-035</t>
+  </si>
+  <si>
+    <t>(21565) 인천광역시 남동구 남동대로 774번길 21(구월동)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 강남구 강남대로 428 만이빌딩 2층</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 강남구 청담동 88-18 1층, 2층</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 서초구 강남대로 453 서초빌딩 4, 5층</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 마포구 양화로 162, 9층 일부(동교동, 좋은사람들빌딩)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 강남구 압구정로 425 4층</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 서초구 강남대로69길 8, 10층 (06611) 서초동, 케이아이타워(KI타워)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Seoul Seocho-gu</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 강남구 언주로 626 논현로얄팰리스 1층 101호</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울시 강남구 역삼동 604-1번지 라이브빌딩 1,2층</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -4367,13 +4393,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>816</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>817</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>818</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -4747,7 +4773,7 @@
     </row>
     <row r="5" spans="1:32" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>28</v>
@@ -4827,7 +4853,7 @@
     </row>
     <row r="6" spans="1:32" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>28</v>
@@ -5028,7 +5054,7 @@
         <v>689</v>
       </c>
       <c r="U8" s="3" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="V8" s="2" t="s">
         <v>690</v>
@@ -5098,7 +5124,9 @@
       <c r="T9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="U9" s="3"/>
+      <c r="U9" s="3" t="s">
+        <v>973</v>
+      </c>
       <c r="V9" s="2" t="s">
         <v>695</v>
       </c>
@@ -5176,7 +5204,9 @@
       <c r="T10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="U10" s="3"/>
+      <c r="U10" s="3" t="s">
+        <v>973</v>
+      </c>
       <c r="V10" s="2" t="s">
         <v>696</v>
       </c>
@@ -5254,7 +5284,9 @@
       <c r="T11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="U11" s="3"/>
+      <c r="U11" s="3" t="s">
+        <v>973</v>
+      </c>
       <c r="V11" s="2" t="s">
         <v>697</v>
       </c>
@@ -5283,25 +5315,25 @@
     </row>
     <row r="12" spans="1:32" ht="132" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>793</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="G12" s="3" t="s">
         <v>794</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>794</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>794</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>795</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>40</v>
@@ -5319,17 +5351,19 @@
         <v>120</v>
       </c>
       <c r="P12" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="U12" s="3" t="s">
+        <v>974</v>
+      </c>
+      <c r="X12" s="11" t="s">
         <v>796</v>
-      </c>
-      <c r="Q12" s="3" t="s">
-        <v>804</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="U12"/>
-      <c r="X12" s="11" t="s">
-        <v>797</v>
       </c>
       <c r="AA12" s="2"/>
       <c r="AB12" s="2" t="s">
@@ -5344,25 +5378,25 @@
     </row>
     <row r="13" spans="1:32" ht="132" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>793</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>794</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>40</v>
@@ -5380,15 +5414,17 @@
         <v>180</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q13" s="9" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="U13"/>
+        <v>689</v>
+      </c>
+      <c r="U13" s="3" t="s">
+        <v>974</v>
+      </c>
       <c r="AA13" s="2"/>
       <c r="AB13" s="2" t="s">
         <v>35</v>
@@ -5402,25 +5438,25 @@
     </row>
     <row r="14" spans="1:32" ht="132" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>793</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>794</v>
-      </c>
       <c r="E14" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>40</v>
@@ -5438,15 +5474,17 @@
         <v>180</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q14" s="9" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="U14"/>
+        <v>689</v>
+      </c>
+      <c r="U14" s="3" t="s">
+        <v>974</v>
+      </c>
       <c r="AA14" s="2"/>
       <c r="AB14" s="2" t="s">
         <v>35</v>
@@ -5458,9 +5496,9 @@
         <v>682</v>
       </c>
     </row>
-    <row r="15" spans="1:32" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>28</v>
@@ -5469,7 +5507,7 @@
         <v>765</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>701</v>
@@ -5511,7 +5549,10 @@
         <v>32</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>56</v>
+        <v>689</v>
+      </c>
+      <c r="U15" s="3" t="s">
+        <v>975</v>
       </c>
       <c r="V15" s="2" t="s">
         <v>32</v>
@@ -5541,9 +5582,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>28</v>
@@ -5552,7 +5593,7 @@
         <v>765</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>701</v>
@@ -5594,7 +5635,10 @@
         <v>32</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>56</v>
+        <v>689</v>
+      </c>
+      <c r="U16" s="3" t="s">
+        <v>975</v>
       </c>
       <c r="V16" s="2" t="s">
         <v>32</v>
@@ -5624,9 +5668,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>28</v>
@@ -5635,7 +5679,7 @@
         <v>765</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>701</v>
@@ -5677,7 +5721,10 @@
         <v>32</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>56</v>
+        <v>689</v>
+      </c>
+      <c r="U17" s="3" t="s">
+        <v>975</v>
       </c>
       <c r="V17" s="2" t="s">
         <v>32</v>
@@ -5709,7 +5756,7 @@
     </row>
     <row r="18" spans="1:32" s="2" customFormat="1" ht="178.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>28</v>
@@ -5718,7 +5765,7 @@
         <v>765</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>705</v>
@@ -5758,6 +5805,9 @@
       </c>
       <c r="T18" s="2" t="s">
         <v>42</v>
+      </c>
+      <c r="U18" s="3" t="s">
+        <v>976</v>
       </c>
       <c r="V18" s="2" t="s">
         <v>63</v>
@@ -5789,7 +5839,7 @@
     </row>
     <row r="19" spans="1:32" s="2" customFormat="1" ht="162.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>28</v>
@@ -5798,7 +5848,7 @@
         <v>765</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>705</v>
@@ -5838,6 +5888,9 @@
       </c>
       <c r="T19" s="2" t="s">
         <v>42</v>
+      </c>
+      <c r="U19" s="3" t="s">
+        <v>976</v>
       </c>
       <c r="V19" s="2" t="s">
         <v>63</v>
@@ -5869,7 +5922,7 @@
     </row>
     <row r="20" spans="1:32" s="2" customFormat="1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>28</v>
@@ -5878,7 +5931,7 @@
         <v>771</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>705</v>
@@ -5919,6 +5972,9 @@
       <c r="T20" s="2" t="s">
         <v>42</v>
       </c>
+      <c r="U20" s="3" t="s">
+        <v>976</v>
+      </c>
       <c r="V20" s="2" t="s">
         <v>63</v>
       </c>
@@ -5947,9 +6003,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>28</v>
@@ -5958,7 +6014,7 @@
         <v>774</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>705</v>
@@ -6002,6 +6058,9 @@
       <c r="T21" s="2" t="s">
         <v>42</v>
       </c>
+      <c r="U21" s="3" t="s">
+        <v>976</v>
+      </c>
       <c r="V21" s="2" t="s">
         <v>63</v>
       </c>
@@ -6030,9 +6089,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:32" s="2" customFormat="1" ht="214.5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>28</v>
@@ -6041,7 +6100,7 @@
         <v>775</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>714</v>
@@ -6088,6 +6147,9 @@
       <c r="T22" s="2" t="s">
         <v>73</v>
       </c>
+      <c r="U22" s="3" t="s">
+        <v>977</v>
+      </c>
       <c r="V22" s="2" t="s">
         <v>74</v>
       </c>
@@ -6116,9 +6178,9 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:32" s="2" customFormat="1" ht="198" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>28</v>
@@ -6127,7 +6189,7 @@
         <v>775</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>714</v>
@@ -6174,6 +6236,9 @@
       <c r="T23" s="2" t="s">
         <v>73</v>
       </c>
+      <c r="U23" s="3" t="s">
+        <v>977</v>
+      </c>
       <c r="V23" s="2" t="s">
         <v>74</v>
       </c>
@@ -6202,9 +6267,9 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>28</v>
@@ -6213,7 +6278,7 @@
         <v>775</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>714</v>
@@ -6259,6 +6324,9 @@
       </c>
       <c r="T24" s="2" t="s">
         <v>73</v>
+      </c>
+      <c r="U24" s="3" t="s">
+        <v>977</v>
       </c>
       <c r="V24" s="2" t="s">
         <v>74</v>
@@ -6290,7 +6358,7 @@
     </row>
     <row r="25" spans="1:32" s="2" customFormat="1" ht="122.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>28</v>
@@ -6299,7 +6367,7 @@
         <v>771</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>715</v>
@@ -6344,7 +6412,10 @@
         <v>32</v>
       </c>
       <c r="T25" s="2" t="s">
-        <v>56</v>
+        <v>689</v>
+      </c>
+      <c r="U25" s="3" t="s">
+        <v>978</v>
       </c>
       <c r="V25" s="2" t="s">
         <v>32</v>
@@ -6374,9 +6445,9 @@
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>28</v>
@@ -6385,7 +6456,7 @@
         <v>775</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>715</v>
@@ -6430,7 +6501,10 @@
         <v>32</v>
       </c>
       <c r="T26" s="2" t="s">
-        <v>56</v>
+        <v>689</v>
+      </c>
+      <c r="U26" s="3" t="s">
+        <v>978</v>
       </c>
       <c r="V26" s="2" t="s">
         <v>32</v>
@@ -6460,9 +6534,9 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:32" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>28</v>
@@ -6471,7 +6545,7 @@
         <v>778</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>715</v>
@@ -6516,7 +6590,10 @@
         <v>32</v>
       </c>
       <c r="T27" s="2" t="s">
-        <v>56</v>
+        <v>689</v>
+      </c>
+      <c r="U27" s="3" t="s">
+        <v>978</v>
       </c>
       <c r="V27" s="2" t="s">
         <v>32</v>
@@ -6548,7 +6625,7 @@
     </row>
     <row r="28" spans="1:32" s="2" customFormat="1" ht="158.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>28</v>
@@ -6557,7 +6634,7 @@
         <v>778</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>715</v>
@@ -6602,7 +6679,10 @@
         <v>32</v>
       </c>
       <c r="T28" s="2" t="s">
-        <v>56</v>
+        <v>689</v>
+      </c>
+      <c r="U28" s="3" t="s">
+        <v>978</v>
       </c>
       <c r="V28" s="2" t="s">
         <v>32</v>
@@ -6634,7 +6714,7 @@
     </row>
     <row r="29" spans="1:32" s="2" customFormat="1" ht="126.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>28</v>
@@ -6643,7 +6723,7 @@
         <v>765</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>720</v>
@@ -6688,7 +6768,10 @@
         <v>32</v>
       </c>
       <c r="T29" s="2" t="s">
-        <v>56</v>
+        <v>980</v>
+      </c>
+      <c r="U29" s="3" t="s">
+        <v>979</v>
       </c>
       <c r="V29" s="2" t="s">
         <v>32</v>
@@ -6715,9 +6798,9 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>28</v>
@@ -6726,7 +6809,7 @@
         <v>765</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>720</v>
@@ -6771,7 +6854,10 @@
         <v>32</v>
       </c>
       <c r="T30" s="2" t="s">
-        <v>56</v>
+        <v>980</v>
+      </c>
+      <c r="U30" s="3" t="s">
+        <v>979</v>
       </c>
       <c r="V30" s="2" t="s">
         <v>32</v>
@@ -6795,9 +6881,9 @@
         <v>163</v>
       </c>
     </row>
-    <row r="31" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>28</v>
@@ -6806,7 +6892,7 @@
         <v>765</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>720</v>
@@ -6851,7 +6937,10 @@
         <v>32</v>
       </c>
       <c r="T31" s="2" t="s">
-        <v>56</v>
+        <v>980</v>
+      </c>
+      <c r="U31" s="3" t="s">
+        <v>979</v>
       </c>
       <c r="V31" s="2" t="s">
         <v>32</v>
@@ -6877,7 +6966,7 @@
     </row>
     <row r="32" spans="1:32" s="2" customFormat="1" ht="214.5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>28</v>
@@ -6886,39 +6975,45 @@
         <v>771</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>940</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>940</v>
-      </c>
-      <c r="F32" s="2" t="s">
+      <c r="G32" s="3" t="s">
         <v>941</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>942</v>
       </c>
       <c r="K32" s="2">
         <v>10000000</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="O32" s="2">
         <v>240</v>
       </c>
       <c r="P32" s="2" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="R32" s="3"/>
       <c r="S32" s="3"/>
+      <c r="T32" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="U32" s="3" t="s">
+        <v>981</v>
+      </c>
       <c r="AE32" s="3"/>
     </row>
     <row r="33" spans="1:31" s="2" customFormat="1" ht="264" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>28</v>
@@ -6927,39 +7022,45 @@
         <v>771</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>940</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>940</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>941</v>
-      </c>
       <c r="G33" s="3" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="K33" s="2">
         <v>30000000</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="O33" s="2">
         <v>360</v>
       </c>
       <c r="P33" s="2" t="s">
+        <v>945</v>
+      </c>
+      <c r="Q33" s="3" t="s">
         <v>946</v>
-      </c>
-      <c r="Q33" s="3" t="s">
-        <v>947</v>
       </c>
       <c r="R33" s="3"/>
       <c r="S33" s="3"/>
+      <c r="T33" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="U33" s="3" t="s">
+        <v>981</v>
+      </c>
       <c r="AE33" s="3"/>
     </row>
     <row r="34" spans="1:31" s="2" customFormat="1" ht="396" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>28</v>
@@ -6968,63 +7069,69 @@
         <v>771</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>940</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>940</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>941</v>
-      </c>
       <c r="G34" s="3" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="K34" s="2">
         <v>50000000</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="O34" s="2">
         <v>300</v>
       </c>
       <c r="P34" s="2" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="R34" s="3"/>
       <c r="S34" s="3"/>
+      <c r="T34" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="U34" s="3" t="s">
+        <v>981</v>
+      </c>
       <c r="AE34" s="3"/>
     </row>
-    <row r="35" spans="1:31" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:31" s="2" customFormat="1" ht="280.5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>804</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>805</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="E35" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>806</v>
       </c>
-      <c r="E35" s="2" t="s">
-        <v>806</v>
-      </c>
-      <c r="F35" s="2" t="s">
+      <c r="G35" s="2" t="s">
         <v>807</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>808</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>721</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="K35" s="2">
         <v>6000000</v>
@@ -7039,48 +7146,51 @@
         <v>53</v>
       </c>
       <c r="Q35" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="R35" s="3" t="s">
         <v>810</v>
-      </c>
-      <c r="R35" s="3" t="s">
-        <v>811</v>
       </c>
       <c r="S35" s="3"/>
       <c r="T35" s="2" t="s">
-        <v>56</v>
+        <v>689</v>
+      </c>
+      <c r="U35" s="3" t="s">
+        <v>982</v>
       </c>
       <c r="X35" s="6" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="AD35" s="3"/>
       <c r="AE35" s="3"/>
     </row>
-    <row r="36" spans="1:31" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:31" s="2" customFormat="1" ht="396" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>804</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>805</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>806</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>806</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>807</v>
-      </c>
       <c r="G36" s="2" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="K36" s="2">
         <v>300000</v>
@@ -7095,10 +7205,16 @@
         <v>53</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="R36" s="3"/>
       <c r="S36" s="3"/>
+      <c r="T36" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="U36" s="3" t="s">
+        <v>982</v>
+      </c>
       <c r="AD36" s="3"/>
       <c r="AE36" s="3"/>
     </row>
@@ -7154,13 +7270,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>816</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>817</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>818</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -7291,13 +7407,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>816</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>817</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>818</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -7392,7 +7508,7 @@
         <v>730</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>745</v>
@@ -7473,7 +7589,7 @@
         <v>730</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>745</v>
@@ -7543,7 +7659,7 @@
         <v>730</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>745</v>
@@ -7613,7 +7729,7 @@
         <v>730</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>746</v>
@@ -7660,7 +7776,7 @@
         <v>730</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>746</v>
@@ -7707,7 +7823,7 @@
         <v>730</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>751</v>
@@ -7784,7 +7900,7 @@
         <v>730</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>751</v>
@@ -7853,16 +7969,16 @@
     </row>
     <row r="9" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>167</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>905</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>906</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>907</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>184</v>
@@ -7945,16 +8061,16 @@
     </row>
     <row r="10" spans="1:32" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>167</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>192</v>
@@ -8037,16 +8153,16 @@
     </row>
     <row r="11" spans="1:32" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>167</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>199</v>
@@ -8129,7 +8245,7 @@
     </row>
     <row r="12" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>167</v>
@@ -8138,7 +8254,7 @@
         <v>205</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>206</v>
@@ -8221,7 +8337,7 @@
     </row>
     <row r="13" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>167</v>
@@ -8230,7 +8346,7 @@
         <v>205</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>215</v>
@@ -8313,7 +8429,7 @@
     </row>
     <row r="14" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>167</v>
@@ -8322,7 +8438,7 @@
         <v>205</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>221</v>
@@ -8405,7 +8521,7 @@
     </row>
     <row r="15" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>167</v>
@@ -8414,7 +8530,7 @@
         <v>205</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>221</v>
@@ -8497,7 +8613,7 @@
     </row>
     <row r="16" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>167</v>
@@ -8506,7 +8622,7 @@
         <v>205</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>231</v>
@@ -8589,7 +8705,7 @@
     </row>
     <row r="17" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>167</v>
@@ -8598,7 +8714,7 @@
         <v>205</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>237</v>
@@ -8681,7 +8797,7 @@
     </row>
     <row r="18" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>167</v>
@@ -8690,7 +8806,7 @@
         <v>205</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>242</v>
@@ -8773,7 +8889,7 @@
     </row>
     <row r="19" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>167</v>
@@ -8782,7 +8898,7 @@
         <v>205</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>249</v>
@@ -8865,7 +8981,7 @@
     </row>
     <row r="20" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>167</v>
@@ -8874,7 +8990,7 @@
         <v>205</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>249</v>
@@ -8957,7 +9073,7 @@
     </row>
     <row r="21" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>167</v>
@@ -8966,7 +9082,7 @@
         <v>205</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>215</v>
@@ -9049,7 +9165,7 @@
     </row>
     <row r="22" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>167</v>
@@ -9058,7 +9174,7 @@
         <v>205</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>261</v>
@@ -9141,7 +9257,7 @@
     </row>
     <row r="23" spans="1:32" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>167</v>
@@ -9150,7 +9266,7 @@
         <v>205</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>266</v>
@@ -9233,7 +9349,7 @@
     </row>
     <row r="24" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>167</v>
@@ -9242,7 +9358,7 @@
         <v>205</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>272</v>
@@ -9325,7 +9441,7 @@
     </row>
     <row r="25" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>167</v>
@@ -9334,7 +9450,7 @@
         <v>205</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>278</v>
@@ -9417,7 +9533,7 @@
     </row>
     <row r="26" spans="1:32" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>167</v>
@@ -9426,7 +9542,7 @@
         <v>205</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>283</v>
@@ -9509,7 +9625,7 @@
     </row>
     <row r="27" spans="1:32" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>167</v>
@@ -9518,7 +9634,7 @@
         <v>288</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>289</v>
@@ -9601,7 +9717,7 @@
     </row>
     <row r="28" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>167</v>
@@ -9610,7 +9726,7 @@
         <v>288</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>296</v>
@@ -9687,7 +9803,7 @@
     </row>
     <row r="29" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>167</v>
@@ -9696,7 +9812,7 @@
         <v>288</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>303</v>
@@ -9773,7 +9889,7 @@
     </row>
     <row r="30" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>167</v>
@@ -9782,7 +9898,7 @@
         <v>288</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>289</v>
@@ -9859,7 +9975,7 @@
     </row>
     <row r="31" spans="1:32" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>167</v>
@@ -9868,7 +9984,7 @@
         <v>288</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>303</v>
@@ -9945,7 +10061,7 @@
     </row>
     <row r="32" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>167</v>
@@ -9954,7 +10070,7 @@
         <v>288</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>320</v>
@@ -10037,7 +10153,7 @@
     </row>
     <row r="33" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>167</v>
@@ -10046,7 +10162,7 @@
         <v>288</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>320</v>
@@ -10129,7 +10245,7 @@
     </row>
     <row r="34" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>167</v>
@@ -10138,7 +10254,7 @@
         <v>288</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>332</v>
@@ -10221,7 +10337,7 @@
     </row>
     <row r="35" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>167</v>
@@ -10230,7 +10346,7 @@
         <v>288</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>340</v>
@@ -10313,7 +10429,7 @@
     </row>
     <row r="36" spans="1:32" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>167</v>
@@ -10322,7 +10438,7 @@
         <v>288</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>347</v>
@@ -10414,7 +10530,7 @@
         <v>354</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>355</v>
@@ -10506,7 +10622,7 @@
         <v>354</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>355</v>
@@ -10598,7 +10714,7 @@
         <v>354</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>367</v>
@@ -10690,7 +10806,7 @@
         <v>354</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>367</v>
@@ -10782,7 +10898,7 @@
         <v>354</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>376</v>
@@ -10874,7 +10990,7 @@
         <v>354</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>376</v>
@@ -10966,7 +11082,7 @@
         <v>354</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>384</v>
@@ -11058,7 +11174,7 @@
         <v>354</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>384</v>
@@ -11150,7 +11266,7 @@
         <v>354</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>390</v>
@@ -11242,7 +11358,7 @@
         <v>354</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>390</v>
@@ -11334,7 +11450,7 @@
         <v>354</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>390</v>
@@ -11417,7 +11533,7 @@
     </row>
     <row r="48" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>167</v>
@@ -11426,7 +11542,7 @@
         <v>354</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>399</v>
@@ -11509,7 +11625,7 @@
     </row>
     <row r="49" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>167</v>
@@ -11518,7 +11634,7 @@
         <v>354</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>399</v>
@@ -11601,7 +11717,7 @@
     </row>
     <row r="50" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>167</v>
@@ -11610,7 +11726,7 @@
         <v>354</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>399</v>
@@ -11693,7 +11809,7 @@
     </row>
     <row r="51" spans="1:32" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>167</v>
@@ -11702,7 +11818,7 @@
         <v>354</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>407</v>
@@ -11785,7 +11901,7 @@
     </row>
     <row r="52" spans="1:32" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>167</v>
@@ -11794,7 +11910,7 @@
         <v>354</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>407</v>
@@ -11877,7 +11993,7 @@
     </row>
     <row r="53" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>167</v>
@@ -11886,7 +12002,7 @@
         <v>354</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>415</v>
@@ -11969,7 +12085,7 @@
     </row>
     <row r="54" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>167</v>
@@ -11978,7 +12094,7 @@
         <v>354</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>422</v>
@@ -12061,7 +12177,7 @@
     </row>
     <row r="55" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>167</v>
@@ -12070,7 +12186,7 @@
         <v>354</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>427</v>
@@ -12153,7 +12269,7 @@
     </row>
     <row r="56" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>167</v>
@@ -12162,7 +12278,7 @@
         <v>354</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>427</v>
@@ -12245,7 +12361,7 @@
     </row>
     <row r="57" spans="1:32" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>167</v>
@@ -12254,7 +12370,7 @@
         <v>354</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>437</v>
@@ -12337,7 +12453,7 @@
     </row>
     <row r="58" spans="1:32" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>167</v>
@@ -12346,7 +12462,7 @@
         <v>354</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>437</v>
@@ -12429,7 +12545,7 @@
     </row>
     <row r="59" spans="1:32" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>167</v>
@@ -12438,7 +12554,7 @@
         <v>354</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>445</v>
@@ -12521,7 +12637,7 @@
     </row>
     <row r="60" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>167</v>
@@ -12530,7 +12646,7 @@
         <v>354</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>451</v>
@@ -12613,7 +12729,7 @@
     </row>
     <row r="61" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>167</v>
@@ -12622,7 +12738,7 @@
         <v>354</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>451</v>
@@ -12705,7 +12821,7 @@
     </row>
     <row r="62" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>167</v>
@@ -12714,7 +12830,7 @@
         <v>354</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>458</v>
@@ -12797,7 +12913,7 @@
     </row>
     <row r="63" spans="1:32" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>167</v>
@@ -12806,7 +12922,7 @@
         <v>354</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>464</v>
@@ -12931,13 +13047,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>816</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>817</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>818</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -13026,7 +13142,7 @@
     </row>
     <row r="2" spans="1:32" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>469</v>
@@ -13317,13 +13433,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>816</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>817</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>818</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -13412,7 +13528,7 @@
     </row>
     <row r="2" spans="1:32" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>480</v>
@@ -13498,7 +13614,7 @@
     </row>
     <row r="3" spans="1:32" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>480</v>
@@ -13584,7 +13700,7 @@
     </row>
     <row r="4" spans="1:32" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>480</v>
@@ -13711,13 +13827,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>816</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>817</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>818</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -13744,7 +13860,7 @@
         <v>8</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>11</v>
@@ -13794,7 +13910,7 @@
     </row>
     <row r="2" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>491</v>
@@ -13862,7 +13978,7 @@
     </row>
     <row r="3" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>491</v>
@@ -13930,7 +14046,7 @@
     </row>
     <row r="4" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>491</v>
@@ -13998,7 +14114,7 @@
     </row>
     <row r="5" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>491</v>
@@ -14066,7 +14182,7 @@
     </row>
     <row r="6" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>491</v>
@@ -14134,7 +14250,7 @@
     </row>
     <row r="7" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>491</v>
@@ -14202,7 +14318,7 @@
     </row>
     <row r="8" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>491</v>
@@ -14270,7 +14386,7 @@
     </row>
     <row r="9" spans="1:28" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>491</v>
@@ -14338,7 +14454,7 @@
     </row>
     <row r="10" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>491</v>
@@ -14406,7 +14522,7 @@
     </row>
     <row r="11" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>491</v>
@@ -14474,7 +14590,7 @@
     </row>
     <row r="12" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>491</v>
@@ -14542,7 +14658,7 @@
     </row>
     <row r="13" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>491</v>
@@ -14610,7 +14726,7 @@
     </row>
     <row r="14" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>491</v>
@@ -14678,7 +14794,7 @@
     </row>
     <row r="15" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>491</v>
@@ -14746,7 +14862,7 @@
     </row>
     <row r="16" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>491</v>
@@ -14814,7 +14930,7 @@
     </row>
     <row r="17" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>491</v>
@@ -14882,7 +14998,7 @@
     </row>
     <row r="18" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>491</v>
@@ -14950,7 +15066,7 @@
     </row>
     <row r="19" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>491</v>
@@ -15018,7 +15134,7 @@
     </row>
     <row r="20" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>491</v>
@@ -15086,7 +15202,7 @@
     </row>
     <row r="21" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>491</v>
@@ -15154,7 +15270,7 @@
     </row>
     <row r="22" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>491</v>
@@ -15222,7 +15338,7 @@
     </row>
     <row r="23" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>491</v>
@@ -15290,7 +15406,7 @@
     </row>
     <row r="24" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>491</v>
@@ -15358,7 +15474,7 @@
     </row>
     <row r="25" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>491</v>
@@ -15426,7 +15542,7 @@
     </row>
     <row r="26" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>491</v>
@@ -15494,7 +15610,7 @@
     </row>
     <row r="27" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>491</v>
@@ -15562,7 +15678,7 @@
     </row>
     <row r="28" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>491</v>
@@ -15630,7 +15746,7 @@
     </row>
     <row r="29" spans="1:28" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>491</v>
@@ -15698,7 +15814,7 @@
     </row>
     <row r="30" spans="1:28" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>491</v>
@@ -15766,7 +15882,7 @@
     </row>
     <row r="31" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>491</v>
@@ -15834,7 +15950,7 @@
     </row>
     <row r="32" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>491</v>
@@ -15902,7 +16018,7 @@
     </row>
     <row r="33" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>491</v>
@@ -15970,7 +16086,7 @@
     </row>
     <row r="34" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>491</v>
@@ -16038,7 +16154,7 @@
     </row>
     <row r="35" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>491</v>
@@ -16106,7 +16222,7 @@
     </row>
     <row r="36" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>491</v>
@@ -16174,7 +16290,7 @@
     </row>
     <row r="37" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>491</v>
@@ -16242,7 +16358,7 @@
     </row>
     <row r="38" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>491</v>
@@ -16310,7 +16426,7 @@
     </row>
     <row r="39" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>491</v>
@@ -16325,7 +16441,7 @@
         <v>494</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>57</v>
@@ -16340,7 +16456,7 @@
         <v>8</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="P39" s="3" t="s">
         <v>495</v>
@@ -16372,7 +16488,7 @@
     </row>
     <row r="40" spans="1:28" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>491</v>
@@ -16387,7 +16503,7 @@
         <v>498</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>32</v>
@@ -16405,7 +16521,7 @@
         <v>10</v>
       </c>
       <c r="O40" s="2" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="P40" s="3" t="s">
         <v>499</v>
@@ -16437,7 +16553,7 @@
     </row>
     <row r="41" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>491</v>
@@ -16508,7 +16624,7 @@
     </row>
     <row r="42" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>491</v>
@@ -16579,7 +16695,7 @@
     </row>
     <row r="43" spans="1:28" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>491</v>
@@ -16594,13 +16710,13 @@
         <v>618</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>32</v>
@@ -16650,7 +16766,7 @@
     </row>
     <row r="44" spans="1:28" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>491</v>
@@ -16665,13 +16781,13 @@
         <v>618</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="H44" s="2" t="s">
+        <v>930</v>
+      </c>
+      <c r="I44" s="2" t="s">
         <v>931</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>932</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>32</v>
@@ -16721,7 +16837,7 @@
     </row>
     <row r="45" spans="1:28" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>491</v>
@@ -16792,7 +16908,7 @@
     </row>
     <row r="46" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>491</v>
@@ -16863,7 +16979,7 @@
     </row>
     <row r="47" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>491</v>
@@ -16934,7 +17050,7 @@
     </row>
     <row r="48" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>491</v>
@@ -17005,7 +17121,7 @@
     </row>
     <row r="49" spans="1:28" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>491</v>
@@ -17076,7 +17192,7 @@
     </row>
     <row r="50" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>491</v>
@@ -17147,7 +17263,7 @@
     </row>
     <row r="51" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>491</v>
@@ -17218,7 +17334,7 @@
     </row>
     <row r="52" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>491</v>
@@ -17289,7 +17405,7 @@
     </row>
     <row r="53" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>491</v>
@@ -17360,7 +17476,7 @@
     </row>
     <row r="54" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>491</v>
@@ -17431,7 +17547,7 @@
     </row>
     <row r="55" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>491</v>
@@ -17502,7 +17618,7 @@
     </row>
     <row r="56" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>491</v>
@@ -17573,7 +17689,7 @@
     </row>
     <row r="57" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>491</v>
@@ -17644,7 +17760,7 @@
     </row>
     <row r="58" spans="1:28" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>491</v>

</xml_diff>